<commit_message>
implementing a metadata approach to mapping instead of having python embedded in the mapping
</commit_message>
<xml_diff>
--- a/mappings/bronze_to_silver/state.xlsx
+++ b/mappings/bronze_to_silver/state.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nason\Desktop\Projects\ActiveProjects\BlixHealth\mappings\bronze_to_silver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B5E684-CCD3-4F7E-86F9-0EE4B14B425F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6A2739-5785-4B5B-8E33-D4AD1943A27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
   <si>
     <t>source_database</t>
   </si>
@@ -96,9 +96,6 @@
     <t>UPPER(TRIM(state_id))</t>
   </si>
   <si>
-    <t>state_id.trim().upper()</t>
-  </si>
-  <si>
     <t>state_name</t>
   </si>
   <si>
@@ -111,7 +108,13 @@
     <t>LEFT(TRIM(county_fips), 2)</t>
   </si>
   <si>
-    <t>county_fips.strip()[:2]</t>
+    <t>trim | upper</t>
+  </si>
+  <si>
+    <t>trim</t>
+  </si>
+  <si>
+    <t>trim | substring:0:2</t>
   </si>
 </sst>
 </file>
@@ -482,6 +485,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -540,6 +552,9 @@
       <c r="I2" t="s">
         <v>17</v>
       </c>
+      <c r="J2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -567,7 +582,7 @@
         <v>19</v>
       </c>
       <c r="J3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -581,7 +596,7 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -590,7 +605,10 @@
         <v>15</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -604,7 +622,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
@@ -613,13 +631,13 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" t="s">
         <v>23</v>
       </c>
-      <c r="I5" t="s">
-        <v>24</v>
-      </c>
       <c r="J5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made changes to DAGs
</commit_message>
<xml_diff>
--- a/mappings/bronze_to_silver/state.xlsx
+++ b/mappings/bronze_to_silver/state.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nason\Desktop\Projects\ActiveProjects\BlixHealth\mappings\bronze_to_silver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6A2739-5785-4B5B-8E33-D4AD1943A27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC5A4048-96C9-4385-A03D-93344796B088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="27">
   <si>
     <t>source_database</t>
   </si>
@@ -490,6 +490,9 @@
     <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.21875" bestFit="1" customWidth="1"/>
@@ -540,6 +543,9 @@
       <c r="C2" t="s">
         <v>13</v>
       </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
       <c r="F2" t="s">
         <v>14</v>
       </c>
@@ -569,6 +575,9 @@
       <c r="D3" t="s">
         <v>16</v>
       </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
@@ -598,6 +607,9 @@
       <c r="D4" t="s">
         <v>20</v>
       </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
       <c r="F4" t="s">
         <v>14</v>
       </c>
@@ -623,6 +635,9 @@
       </c>
       <c r="D5" t="s">
         <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>

</xml_diff>